<commit_message>
Pyramid of Khafre update
This version extends the original Khufu (G1) implementation to the
Pyramid of Khafre (G2).
</commit_message>
<xml_diff>
--- a/AdditionalData/Tables/Height just before changes in thickness thickness corrected.xlsx
+++ b/AdditionalData/Tables/Height just before changes in thickness thickness corrected.xlsx
@@ -195,7 +195,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -610,9 +610,7 @@
       <c r="M4" s="4"/>
       <c r="N4" s="4"/>
       <c r="O4" s="4"/>
-      <c r="P4" s="1" t="n">
-        <v>26.98</v>
-      </c>
+      <c r="P4" s="1"/>
       <c r="Q4" s="4" t="n">
         <v>27.69</v>
       </c>
@@ -1106,7 +1104,7 @@
         <v>2</v>
       </c>
       <c r="P18" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q18" s="2" t="n">
         <v>4</v>

</xml_diff>